<commit_message>
creating MX 4.0.4 develop
</commit_message>
<xml_diff>
--- a/InputData/bldgs/BFoCSbQL/BAU Frac of Components Sold by Quality Lvl.xlsx
+++ b/InputData/bldgs/BFoCSbQL/BAU Frac of Components Sold by Quality Lvl.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28609"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Meghan\Dropbox (Energy Innovation)\EPS Versions\eps-1.5.0-us-wipI\InputData\bldgs\BFoCSbQL\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_F50668454FCCA58402D46AFEBF662C7C7DFD7C73" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="120" yWindow="105" windowWidth="20115" windowHeight="9780"/>
+    <workbookView xWindow="120" yWindow="105" windowWidth="20115" windowHeight="9780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -18,264 +19,280 @@
     <sheet name="BFoCSbQL-rural-residential" sheetId="5" r:id="rId4"/>
     <sheet name="BFoCSbQL-commercial" sheetId="4" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191028"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="81">
   <si>
+    <t>BFoCSbQL BAU Fraction of Components Sold by Quality Level</t>
+  </si>
+  <si>
     <t>Source:</t>
   </si>
   <si>
     <t>U.S. Department of Energy</t>
   </si>
   <si>
+    <t>Buildings Energy Data Book (2011 edition)</t>
+  </si>
+  <si>
+    <t>See next tab for table numbers and links</t>
+  </si>
+  <si>
+    <t>Notes:</t>
+  </si>
+  <si>
+    <t>This variable captures what BAU fraction of new building components qualify</t>
+  </si>
+  <si>
+    <t>for energy efficient rebates.</t>
+  </si>
+  <si>
+    <t>Since we do not have data for envelope components, we assume the fraction</t>
+  </si>
+  <si>
+    <t>is the average of the fractions of the "heating" and "cooling and ventilation"</t>
+  </si>
+  <si>
+    <t>components.</t>
+  </si>
+  <si>
+    <t>For the U.S., we use the same fractions for urban residential and rural residential.</t>
+  </si>
+  <si>
+    <t>The table below includes the most important/relevant elements for each subscript, taken from a variety of tables</t>
+  </si>
+  <si>
+    <t>in the DOE Buildings Energy Data Book.  Generally, items with high sales figures and low energy consumption are excluded,</t>
+  </si>
+  <si>
+    <t>so they do not dominate the ENERGY STAR compliance fraction calculation.</t>
+  </si>
+  <si>
+    <t>For instance, cooling and ventilation is based on major system components (central AC, heat pumps), rather than fans.</t>
+  </si>
+  <si>
+    <t>Another example is the exclusion of external power supplies (power strips) from the "Other" category.</t>
+  </si>
+  <si>
+    <t>Subscript</t>
+  </si>
+  <si>
+    <t>Component</t>
+  </si>
+  <si>
+    <t>Shipments</t>
+  </si>
+  <si>
+    <t>ENERGY STAR fraction</t>
+  </si>
+  <si>
+    <t>Table Reference</t>
+  </si>
+  <si>
+    <t>URL</t>
+  </si>
+  <si>
+    <t>heating</t>
+  </si>
+  <si>
+    <t>Gas Furnaces</t>
+  </si>
+  <si>
+    <t>9.1.11</t>
+  </si>
+  <si>
+    <t>http://buildingsdatabook.eren.doe.gov/docs/xls_pdf/9.1.11.xlsx</t>
+  </si>
+  <si>
+    <t>Gas Boilers</t>
+  </si>
+  <si>
+    <t>Oil Boilers</t>
+  </si>
+  <si>
+    <t>Oil Furnaces</t>
+  </si>
+  <si>
+    <t>cooling and ventilation</t>
+  </si>
+  <si>
+    <t>Central AC</t>
+  </si>
+  <si>
+    <t>9.1.10</t>
+  </si>
+  <si>
+    <t>http://buildingsdatabook.eren.doe.gov/docs/xls_pdf/9.1.10.xlsx</t>
+  </si>
+  <si>
+    <t>Air-Source Heat Pumps</t>
+  </si>
+  <si>
+    <t>Geothermal Heat Pumps</t>
+  </si>
+  <si>
     <t>lighting</t>
   </si>
   <si>
+    <t>Medium Screw-Base Lamps</t>
+  </si>
+  <si>
+    <t>9.1.9</t>
+  </si>
+  <si>
+    <t>http://buildingsdatabook.eren.doe.gov/docs/xls_pdf/9.1.9.xlsx</t>
+  </si>
+  <si>
+    <t>appliances (residential)</t>
+  </si>
+  <si>
+    <t>dishwashers</t>
+  </si>
+  <si>
+    <t>9.1.8</t>
+  </si>
+  <si>
+    <t>http://buildingsdatabook.eren.doe.gov/docs/xls_pdf/9.1.8.xlsx</t>
+  </si>
+  <si>
+    <t>refrigerators</t>
+  </si>
+  <si>
+    <t>clothes washers</t>
+  </si>
+  <si>
+    <t>appliances (commercial)</t>
+  </si>
+  <si>
+    <t>commercial refrigeration</t>
+  </si>
+  <si>
+    <t>9.1.12</t>
+  </si>
+  <si>
+    <t>http://buildingsdatabook.eren.doe.gov/docs/xls_pdf/9.1.12.xlsx</t>
+  </si>
+  <si>
+    <t>commercial steam cookers</t>
+  </si>
+  <si>
+    <t>bottled water coolers</t>
+  </si>
+  <si>
+    <t>commercial dishwashers</t>
+  </si>
+  <si>
+    <t>ice machines</t>
+  </si>
+  <si>
+    <t>commercial fryers</t>
+  </si>
+  <si>
+    <t>hot food holding cabinets</t>
+  </si>
+  <si>
+    <t>cold beverage vending machines</t>
+  </si>
+  <si>
+    <t>other (residential)</t>
+  </si>
+  <si>
+    <t>TV</t>
+  </si>
+  <si>
+    <t>9.1.13</t>
+  </si>
+  <si>
+    <t>http://buildingsdatabook.eren.doe.gov/docs/xls_pdf/9.1.13.xlsx</t>
+  </si>
+  <si>
+    <t>telephony</t>
+  </si>
+  <si>
+    <t>DVD/VCR</t>
+  </si>
+  <si>
+    <t>audio/video</t>
+  </si>
+  <si>
+    <t>battery charging system</t>
+  </si>
+  <si>
+    <t>other (commercial)</t>
+  </si>
+  <si>
+    <t>computers</t>
+  </si>
+  <si>
+    <t>9.1.14</t>
+  </si>
+  <si>
+    <t>http://buildingsdatabook.eren.doe.gov/docs/xls_pdf/9.1.14.xlsx</t>
+  </si>
+  <si>
+    <t>monitors</t>
+  </si>
+  <si>
+    <t>printers</t>
+  </si>
+  <si>
+    <t>fascimile</t>
+  </si>
+  <si>
+    <t>copiers</t>
+  </si>
+  <si>
+    <t>scanners</t>
+  </si>
+  <si>
+    <t>multi-function devices</t>
+  </si>
+  <si>
+    <t>Dimensionless fraction of total components</t>
+  </si>
+  <si>
+    <t>standard-compliant</t>
+  </si>
+  <si>
+    <t>rebate-qualifying</t>
+  </si>
+  <si>
+    <t>envelope</t>
+  </si>
+  <si>
     <t>appliances</t>
   </si>
   <si>
     <t>other</t>
-  </si>
-  <si>
-    <t>Subscript</t>
-  </si>
-  <si>
-    <t>Component</t>
-  </si>
-  <si>
-    <t>ENERGY STAR fraction</t>
-  </si>
-  <si>
-    <t>Table Reference</t>
-  </si>
-  <si>
-    <t>URL</t>
-  </si>
-  <si>
-    <t>Central AC</t>
-  </si>
-  <si>
-    <t>9.1.10</t>
-  </si>
-  <si>
-    <t>http://buildingsdatabook.eren.doe.gov/docs/xls_pdf/9.1.10.xlsx</t>
-  </si>
-  <si>
-    <t>Air-Source Heat Pumps</t>
-  </si>
-  <si>
-    <t>Geothermal Heat Pumps</t>
-  </si>
-  <si>
-    <t>Gas Furnaces</t>
-  </si>
-  <si>
-    <t>Gas Boilers</t>
-  </si>
-  <si>
-    <t>Oil Boilers</t>
-  </si>
-  <si>
-    <t>Oil Furnaces</t>
-  </si>
-  <si>
-    <t>9.1.11</t>
-  </si>
-  <si>
-    <t>http://buildingsdatabook.eren.doe.gov/docs/xls_pdf/9.1.11.xlsx</t>
-  </si>
-  <si>
-    <t>Shipments</t>
-  </si>
-  <si>
-    <t>9.1.12</t>
-  </si>
-  <si>
-    <t>Medium Screw-Base Lamps</t>
-  </si>
-  <si>
-    <t>9.1.9</t>
-  </si>
-  <si>
-    <t>http://buildingsdatabook.eren.doe.gov/docs/xls_pdf/9.1.9.xlsx</t>
-  </si>
-  <si>
-    <t>dishwashers</t>
-  </si>
-  <si>
-    <t>refrigerators</t>
-  </si>
-  <si>
-    <t>clothes washers</t>
-  </si>
-  <si>
-    <t>9.1.8</t>
-  </si>
-  <si>
-    <t>http://buildingsdatabook.eren.doe.gov/docs/xls_pdf/9.1.8.xlsx</t>
-  </si>
-  <si>
-    <t>other (commercial)</t>
-  </si>
-  <si>
-    <t>commercial refrigeration</t>
-  </si>
-  <si>
-    <t>hot food holding cabinets</t>
-  </si>
-  <si>
-    <t>commercial steam cookers</t>
-  </si>
-  <si>
-    <t>cold beverage vending machines</t>
-  </si>
-  <si>
-    <t>bottled water coolers</t>
-  </si>
-  <si>
-    <t>appliances (residential)</t>
-  </si>
-  <si>
-    <t>appliances (commercial)</t>
-  </si>
-  <si>
-    <t>http://buildingsdatabook.eren.doe.gov/docs/xls_pdf/9.1.12.xlsx</t>
-  </si>
-  <si>
-    <t>commercial dishwashers</t>
-  </si>
-  <si>
-    <t>ice machines</t>
-  </si>
-  <si>
-    <t>commercial fryers</t>
-  </si>
-  <si>
-    <t>other (residential)</t>
-  </si>
-  <si>
-    <t>TV</t>
-  </si>
-  <si>
-    <t>telephony</t>
-  </si>
-  <si>
-    <t>DVD/VCR</t>
-  </si>
-  <si>
-    <t>audio/video</t>
-  </si>
-  <si>
-    <t>battery charging system</t>
-  </si>
-  <si>
-    <t>The table below includes the most important/relevant elements for each subscript, taken from a variety of tables</t>
-  </si>
-  <si>
-    <t>in the DOE Buildings Energy Data Book.  Generally, items with high sales figures and low energy consumption are excluded,</t>
-  </si>
-  <si>
-    <t>so they do not dominate the ENERGY STAR compliance fraction calculation.</t>
-  </si>
-  <si>
-    <t>Another example is the exclusion of external power supplies (power strips) from the "Other" category.</t>
-  </si>
-  <si>
-    <t>9.1.13</t>
-  </si>
-  <si>
-    <t>http://buildingsdatabook.eren.doe.gov/docs/xls_pdf/9.1.13.xlsx</t>
-  </si>
-  <si>
-    <t>computers</t>
-  </si>
-  <si>
-    <t>monitors</t>
-  </si>
-  <si>
-    <t>printers</t>
-  </si>
-  <si>
-    <t>fascimile</t>
-  </si>
-  <si>
-    <t>copiers</t>
-  </si>
-  <si>
-    <t>scanners</t>
-  </si>
-  <si>
-    <t>multi-function devices</t>
-  </si>
-  <si>
-    <t>9.1.14</t>
-  </si>
-  <si>
-    <t>http://buildingsdatabook.eren.doe.gov/docs/xls_pdf/9.1.14.xlsx</t>
-  </si>
-  <si>
-    <t>BFoCSbQL BAU Fraction of Components Sold by Quality Level</t>
-  </si>
-  <si>
-    <t>cooling and ventilation</t>
-  </si>
-  <si>
-    <t>heating</t>
-  </si>
-  <si>
-    <t>envelope</t>
-  </si>
-  <si>
-    <t>standard-compliant</t>
-  </si>
-  <si>
-    <t>rebate-qualifying</t>
-  </si>
-  <si>
-    <t>For instance, cooling and ventilation is based on major system components (central AC, heat pumps), rather than fans.</t>
-  </si>
-  <si>
-    <t>Notes:</t>
-  </si>
-  <si>
-    <t>Since we do not have data for envelope components, we assume the fraction</t>
-  </si>
-  <si>
-    <t>is the average of the fractions of the "heating" and "cooling and ventilation"</t>
-  </si>
-  <si>
-    <t>components.</t>
-  </si>
-  <si>
-    <t>Buildings Energy Data Book (2011 edition)</t>
-  </si>
-  <si>
-    <t>See next tab for table numbers and links</t>
-  </si>
-  <si>
-    <t>For the U.S., we use the same fractions for urban residential and rural residential.</t>
-  </si>
-  <si>
-    <t>Dimensionless fraction of total components</t>
-  </si>
-  <si>
-    <t>This variable captures what BAU fraction of new building components qualify</t>
-  </si>
-  <si>
-    <t>for energy efficient rebates.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -350,7 +367,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -371,16 +388,11 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -400,9 +412,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -440,9 +452,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -477,7 +489,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -512,7 +524,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -685,75 +697,75 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
     <col min="2" max="2" width="54.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
       <c r="B4" s="2">
         <v>2012</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2">
       <c r="B5" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
       <c r="B6" s="6" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="17" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="17" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
       <c r="A15" t="s">
-        <v>77</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -763,9 +775,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F38"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="31" customWidth="1"/>
@@ -775,57 +787,57 @@
     <col min="6" max="6" width="59.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
       <c r="A7" s="3" t="s">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="C7" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>8</v>
-      </c>
       <c r="F7" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>66</v>
+        <v>23</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="C8" s="2">
         <v>2197000</v>
@@ -834,15 +846,15 @@
         <v>0.61</v>
       </c>
       <c r="E8" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
       <c r="B9" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="C9" s="2">
         <v>192000</v>
@@ -851,15 +863,15 @@
         <v>0.52</v>
       </c>
       <c r="E9" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
       <c r="B10" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="C10" s="2">
         <v>123000</v>
@@ -868,16 +880,16 @@
         <v>0.61</v>
       </c>
       <c r="E10" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
       <c r="A11" s="7"/>
       <c r="B11" s="7" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="C11" s="8">
         <v>56000</v>
@@ -886,54 +898,53 @@
         <v>0.36</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="B12" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="C12" s="13">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" s="2">
         <v>3519000</v>
       </c>
-      <c r="D12" s="13">
+      <c r="D12" s="2">
         <v>0.27</v>
       </c>
-      <c r="E12" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="F12" s="14" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="12"/>
-      <c r="B13" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="C13" s="13">
+      <c r="E12" t="s">
+        <v>32</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="B13" t="s">
+        <v>34</v>
+      </c>
+      <c r="C13" s="2">
         <v>1652000</v>
       </c>
-      <c r="D13" s="13">
+      <c r="D13" s="2">
         <v>0.46</v>
       </c>
-      <c r="E13" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="F13" s="14" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E13" t="s">
+        <v>32</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
       <c r="A14" s="7"/>
       <c r="B14" s="7" t="s">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="C14" s="8">
         <v>128000</v>
@@ -942,18 +953,18 @@
         <v>0.47</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
       <c r="A15" s="7" t="s">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="C15" s="8">
         <v>1658000</v>
@@ -962,18 +973,18 @@
         <v>0.2</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B16" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="C16" s="2">
         <f>5.6*10^6</f>
@@ -983,15 +994,15 @@
         <v>1</v>
       </c>
       <c r="E16" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
       <c r="B17" t="s">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="C17" s="2">
         <f>9.4*10^6</f>
@@ -1001,15 +1012,15 @@
         <v>0.5</v>
       </c>
       <c r="E17" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
       <c r="B18" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="C18" s="2">
         <f>8.2*10^6</f>
@@ -1019,18 +1030,18 @@
         <v>0.64</v>
       </c>
       <c r="E18" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="B19" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="C19" s="2">
         <v>317000</v>
@@ -1039,15 +1050,15 @@
         <v>0.72</v>
       </c>
       <c r="E19" t="s">
-        <v>22</v>
+        <v>48</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
       <c r="B20" t="s">
-        <v>34</v>
+        <v>50</v>
       </c>
       <c r="C20" s="2">
         <v>14000</v>
@@ -1056,15 +1067,15 @@
         <v>0.35</v>
       </c>
       <c r="E20" t="s">
-        <v>22</v>
+        <v>48</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
       <c r="B21" t="s">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="C21" s="2">
         <v>1454000</v>
@@ -1073,15 +1084,15 @@
         <v>0.43</v>
       </c>
       <c r="E21" t="s">
-        <v>22</v>
+        <v>48</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
       <c r="B22" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="C22" s="2">
         <v>38000</v>
@@ -1090,15 +1101,15 @@
         <v>0.74</v>
       </c>
       <c r="E22" t="s">
-        <v>22</v>
+        <v>48</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
       <c r="B23" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="C23" s="2">
         <v>111000</v>
@@ -1107,15 +1118,15 @@
         <v>0.63</v>
       </c>
       <c r="E23" t="s">
-        <v>22</v>
+        <v>48</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
       <c r="B24" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C24" s="2">
         <v>84000</v>
@@ -1124,15 +1135,15 @@
         <v>0.19</v>
       </c>
       <c r="E24" t="s">
-        <v>22</v>
+        <v>48</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
       <c r="B25" t="s">
-        <v>33</v>
+        <v>55</v>
       </c>
       <c r="C25" s="2">
         <v>37000</v>
@@ -1141,16 +1152,16 @@
         <v>0.63</v>
       </c>
       <c r="E25" t="s">
-        <v>22</v>
+        <v>48</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
       <c r="A26" s="7"/>
       <c r="B26" s="7" t="s">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="C26" s="8">
         <v>243000</v>
@@ -1159,18 +1170,18 @@
         <v>0.28000000000000003</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>22</v>
+        <v>48</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
       <c r="A27" t="s">
-        <v>43</v>
+        <v>57</v>
       </c>
       <c r="B27" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="C27" s="2">
         <v>42743000</v>
@@ -1179,15 +1190,15 @@
         <v>0.8</v>
       </c>
       <c r="E27" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
       <c r="B28" t="s">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="C28" s="2">
         <v>28656</v>
@@ -1196,15 +1207,15 @@
         <v>0.68</v>
       </c>
       <c r="E28" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
       <c r="B29" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="C29" s="2">
         <v>1684000</v>
@@ -1213,15 +1224,15 @@
         <v>0.67</v>
       </c>
       <c r="E29" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
       <c r="B30" t="s">
-        <v>47</v>
+        <v>63</v>
       </c>
       <c r="C30" s="2">
         <v>32919000</v>
@@ -1230,15 +1241,15 @@
         <v>0.35</v>
       </c>
       <c r="E30" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
       <c r="B31" t="s">
-        <v>48</v>
+        <v>64</v>
       </c>
       <c r="C31" s="2">
         <v>42674000</v>
@@ -1247,18 +1258,18 @@
         <v>0.34</v>
       </c>
       <c r="E31" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
       <c r="A32" t="s">
-        <v>31</v>
+        <v>65</v>
       </c>
       <c r="B32" t="s">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="C32" s="2">
         <f>69.5*10^6</f>
@@ -1268,15 +1279,15 @@
         <v>0.71</v>
       </c>
       <c r="E32" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="33" spans="2:6">
       <c r="B33" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="C33" s="2">
         <f>28.2*10^6</f>
@@ -1286,15 +1297,15 @@
         <v>0.43</v>
       </c>
       <c r="E33" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="34" spans="2:6">
       <c r="B34" t="s">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="C34" s="2">
         <f>7.8*10^6</f>
@@ -1304,15 +1315,15 @@
         <v>0.99</v>
       </c>
       <c r="E34" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="35" spans="2:6">
       <c r="B35" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
       <c r="C35" s="2">
         <f>3.7*10^6</f>
@@ -1322,15 +1333,15 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="E35" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="36" spans="2:6">
       <c r="B36" t="s">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="C36" s="2">
         <f>0.2*10^6</f>
@@ -1340,15 +1351,15 @@
         <v>0.79</v>
       </c>
       <c r="E36" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="37" spans="2:6" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="37" spans="2:6">
       <c r="B37" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="C37" s="2">
         <f>0.7*10^6</f>
@@ -1358,15 +1369,15 @@
         <v>0.99</v>
       </c>
       <c r="E37" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="38" spans="2:6">
       <c r="B38" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="C38" s="2">
         <f>20.2*10^6</f>
@@ -1376,66 +1387,66 @@
         <v>0.99</v>
       </c>
       <c r="E38" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F12" r:id="rId1"/>
-    <hyperlink ref="F8" r:id="rId2"/>
-    <hyperlink ref="F13" r:id="rId3"/>
-    <hyperlink ref="F14" r:id="rId4"/>
-    <hyperlink ref="F9" r:id="rId5"/>
-    <hyperlink ref="F10" r:id="rId6"/>
-    <hyperlink ref="F11" r:id="rId7"/>
-    <hyperlink ref="F15" r:id="rId8"/>
-    <hyperlink ref="F16" r:id="rId9"/>
-    <hyperlink ref="F17:F18" r:id="rId10" display="http://buildingsdatabook.eren.doe.gov/docs/xls_pdf/9.1.8.xlsx"/>
-    <hyperlink ref="F19" r:id="rId11"/>
-    <hyperlink ref="F27" r:id="rId12"/>
-    <hyperlink ref="F28:F31" r:id="rId13" display="http://buildingsdatabook.eren.doe.gov/docs/xls_pdf/9.1.13.xlsx"/>
-    <hyperlink ref="F20" r:id="rId14"/>
-    <hyperlink ref="F21" r:id="rId15"/>
-    <hyperlink ref="F25" r:id="rId16"/>
-    <hyperlink ref="F26" r:id="rId17"/>
-    <hyperlink ref="F22" r:id="rId18"/>
-    <hyperlink ref="F23" r:id="rId19"/>
-    <hyperlink ref="F24" r:id="rId20"/>
+    <hyperlink ref="F12" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
+    <hyperlink ref="F8" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
+    <hyperlink ref="F13" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
+    <hyperlink ref="F14" r:id="rId4" xr:uid="{00000000-0004-0000-0100-000003000000}"/>
+    <hyperlink ref="F9" r:id="rId5" xr:uid="{00000000-0004-0000-0100-000004000000}"/>
+    <hyperlink ref="F10" r:id="rId6" xr:uid="{00000000-0004-0000-0100-000005000000}"/>
+    <hyperlink ref="F11" r:id="rId7" xr:uid="{00000000-0004-0000-0100-000006000000}"/>
+    <hyperlink ref="F15" r:id="rId8" xr:uid="{00000000-0004-0000-0100-000007000000}"/>
+    <hyperlink ref="F16" r:id="rId9" xr:uid="{00000000-0004-0000-0100-000008000000}"/>
+    <hyperlink ref="F17:F18" r:id="rId10" display="http://buildingsdatabook.eren.doe.gov/docs/xls_pdf/9.1.8.xlsx" xr:uid="{00000000-0004-0000-0100-000009000000}"/>
+    <hyperlink ref="F19" r:id="rId11" xr:uid="{00000000-0004-0000-0100-00000A000000}"/>
+    <hyperlink ref="F27" r:id="rId12" xr:uid="{00000000-0004-0000-0100-00000B000000}"/>
+    <hyperlink ref="F28:F31" r:id="rId13" display="http://buildingsdatabook.eren.doe.gov/docs/xls_pdf/9.1.13.xlsx" xr:uid="{00000000-0004-0000-0100-00000C000000}"/>
+    <hyperlink ref="F20" r:id="rId14" xr:uid="{00000000-0004-0000-0100-00000D000000}"/>
+    <hyperlink ref="F21" r:id="rId15" xr:uid="{00000000-0004-0000-0100-00000E000000}"/>
+    <hyperlink ref="F25" r:id="rId16" xr:uid="{00000000-0004-0000-0100-00000F000000}"/>
+    <hyperlink ref="F26" r:id="rId17" xr:uid="{00000000-0004-0000-0100-000010000000}"/>
+    <hyperlink ref="F22" r:id="rId18" xr:uid="{00000000-0004-0000-0100-000011000000}"/>
+    <hyperlink ref="F23" r:id="rId19" xr:uid="{00000000-0004-0000-0100-000012000000}"/>
+    <hyperlink ref="F24" r:id="rId20" xr:uid="{00000000-0004-0000-0100-000013000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28.85546875" customWidth="1"/>
     <col min="2" max="2" width="20.85546875" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
-        <v>78</v>
+    <row r="1" spans="1:3" ht="30">
+      <c r="A1" s="14" t="s">
+        <v>75</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>66</v>
+        <v>23</v>
       </c>
       <c r="B2" s="11">
         <f>1-C2</f>
@@ -1446,9 +1457,9 @@
         <v>0.59781931464174454</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="B3" s="11">
         <f t="shared" ref="B3:B7" si="0">1-C3</f>
@@ -1459,22 +1470,22 @@
         <v>0.27</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>67</v>
-      </c>
-      <c r="B4" s="15">
+        <v>78</v>
+      </c>
+      <c r="B4" s="13">
         <f t="shared" si="0"/>
         <v>0.56609034267912772</v>
       </c>
-      <c r="C4" s="15">
+      <c r="C4" s="13">
         <f>AVERAGE(C2:C3)</f>
         <v>0.43390965732087228</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="B5" s="11">
         <f t="shared" si="0"/>
@@ -1485,9 +1496,9 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>3</v>
+        <v>79</v>
       </c>
       <c r="B6" s="11">
         <f t="shared" si="0"/>
@@ -1498,9 +1509,9 @@
         <v>0.67017241379310344</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>4</v>
+        <v>80</v>
       </c>
       <c r="B7" s="11">
         <f t="shared" si="0"/>
@@ -1521,32 +1532,32 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28.85546875" customWidth="1"/>
     <col min="2" max="2" width="20.85546875" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
-        <v>78</v>
+    <row r="1" spans="1:3" ht="30">
+      <c r="A1" s="14" t="s">
+        <v>75</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>66</v>
+        <v>23</v>
       </c>
       <c r="B2" s="11">
         <f>1-C2</f>
@@ -1557,9 +1568,9 @@
         <v>0.59781931464174454</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="B3" s="11">
         <f t="shared" ref="B3:B7" si="0">1-C3</f>
@@ -1570,22 +1581,22 @@
         <v>0.27</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>67</v>
-      </c>
-      <c r="B4" s="15">
+        <v>78</v>
+      </c>
+      <c r="B4" s="13">
         <f t="shared" si="0"/>
         <v>0.56609034267912772</v>
       </c>
-      <c r="C4" s="15">
+      <c r="C4" s="13">
         <f>AVERAGE(C2:C3)</f>
         <v>0.43390965732087228</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="B5" s="11">
         <f t="shared" si="0"/>
@@ -1596,9 +1607,9 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>3</v>
+        <v>79</v>
       </c>
       <c r="B6" s="11">
         <f t="shared" si="0"/>
@@ -1609,9 +1620,9 @@
         <v>0.67017241379310344</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>4</v>
+        <v>80</v>
       </c>
       <c r="B7" s="11">
         <f t="shared" si="0"/>
@@ -1629,32 +1640,32 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28.85546875" customWidth="1"/>
     <col min="2" max="2" width="20.85546875" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
-        <v>78</v>
+    <row r="1" spans="1:3" ht="30">
+      <c r="A1" s="14" t="s">
+        <v>75</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>66</v>
+        <v>23</v>
       </c>
       <c r="B2" s="11">
         <f>1-C2</f>
@@ -1665,9 +1676,9 @@
         <v>0.59781931464174454</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="B3" s="11">
         <f t="shared" ref="B3:B7" si="0">1-C3</f>
@@ -1678,22 +1689,22 @@
         <v>0.27</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>67</v>
-      </c>
-      <c r="B4" s="15">
+        <v>78</v>
+      </c>
+      <c r="B4" s="13">
         <f t="shared" si="0"/>
         <v>0.56609034267912772</v>
       </c>
-      <c r="C4" s="15">
+      <c r="C4" s="13">
         <f>AVERAGE(C2:C3)</f>
         <v>0.43390965732087228</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="B5" s="11">
         <f t="shared" si="0"/>
@@ -1704,9 +1715,9 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>3</v>
+        <v>79</v>
       </c>
       <c r="B6" s="11">
         <f t="shared" si="0"/>
@@ -1717,9 +1728,9 @@
         <v>0.46288946910356832</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>4</v>
+        <v>80</v>
       </c>
       <c r="B7" s="11">
         <f t="shared" si="0"/>
@@ -1737,4 +1748,175 @@
     <ignoredError sqref="C2:C3 C5:C7" formulaRange="1"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009A9DAB439B36DB4795F39C4E722C7BC4" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="44674c89fa9bc5e97a878a6680c46188">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="79748b23-d81a-423e-9112-21109dc864e6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="447839a363ea5a12024b5bf1ab53ed90" ns2:_="">
+    <xsd:import namespace="79748b23-d81a-423e-9112-21109dc864e6"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="79748b23-d81a-423e-9112-21109dc864e6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B4FA29A-46AB-4247-BFBB-656DB271D58F}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7A76A8DF-0475-4A58-9E12-A558E763ED54}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D4A9E4D-1172-44F3-A410-61C78A33C523}"/>
 </file>
</xml_diff>